<commit_message>
forward: update frozen E16 E18 E21 real-open ledgers
</commit_message>
<xml_diff>
--- a/forward/e21/E21_forward_dashboard.xlsx
+++ b/forward/e21/E21_forward_dashboard.xlsx
@@ -416,7 +416,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:W16"/>
+  <dimension ref="A1:AE17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -533,6 +533,46 @@
       <c r="W1" t="inlineStr">
         <is>
           <t>e45_exposure</t>
+        </is>
+      </c>
+      <c r="X1" t="inlineStr">
+        <is>
+          <t>fuse_additive</t>
+        </is>
+      </c>
+      <c r="Y1" t="inlineStr">
+        <is>
+          <t>dh_exposure_live</t>
+        </is>
+      </c>
+      <c r="Z1" t="inlineStr">
+        <is>
+          <t>dh_id</t>
+        </is>
+      </c>
+      <c r="AA1" t="inlineStr">
+        <is>
+          <t>dh_exposure</t>
+        </is>
+      </c>
+      <c r="AB1" t="inlineStr">
+        <is>
+          <t>e16_financial_pre_dh</t>
+        </is>
+      </c>
+      <c r="AC1" t="inlineStr">
+        <is>
+          <t>e16_telecom_pre_dh</t>
+        </is>
+      </c>
+      <c r="AD1" t="inlineStr">
+        <is>
+          <t>e16_0050_pre_dh</t>
+        </is>
+      </c>
+      <c r="AE1" t="inlineStr">
+        <is>
+          <t>live_cutover_ballot</t>
         </is>
       </c>
     </row>
@@ -602,6 +642,14 @@
       <c r="U2" t="inlineStr"/>
       <c r="V2" t="inlineStr"/>
       <c r="W2" t="inlineStr"/>
+      <c r="X2" t="inlineStr"/>
+      <c r="Y2" t="inlineStr"/>
+      <c r="Z2" t="inlineStr"/>
+      <c r="AA2" t="inlineStr"/>
+      <c r="AB2" t="inlineStr"/>
+      <c r="AC2" t="inlineStr"/>
+      <c r="AD2" t="inlineStr"/>
+      <c r="AE2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -669,6 +717,14 @@
       <c r="U3" t="inlineStr"/>
       <c r="V3" t="inlineStr"/>
       <c r="W3" t="inlineStr"/>
+      <c r="X3" t="inlineStr"/>
+      <c r="Y3" t="inlineStr"/>
+      <c r="Z3" t="inlineStr"/>
+      <c r="AA3" t="inlineStr"/>
+      <c r="AB3" t="inlineStr"/>
+      <c r="AC3" t="inlineStr"/>
+      <c r="AD3" t="inlineStr"/>
+      <c r="AE3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -736,6 +792,14 @@
       <c r="U4" t="inlineStr"/>
       <c r="V4" t="inlineStr"/>
       <c r="W4" t="inlineStr"/>
+      <c r="X4" t="inlineStr"/>
+      <c r="Y4" t="inlineStr"/>
+      <c r="Z4" t="inlineStr"/>
+      <c r="AA4" t="inlineStr"/>
+      <c r="AB4" t="inlineStr"/>
+      <c r="AC4" t="inlineStr"/>
+      <c r="AD4" t="inlineStr"/>
+      <c r="AE4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -803,6 +867,14 @@
       <c r="U5" t="inlineStr"/>
       <c r="V5" t="inlineStr"/>
       <c r="W5" t="inlineStr"/>
+      <c r="X5" t="inlineStr"/>
+      <c r="Y5" t="inlineStr"/>
+      <c r="Z5" t="inlineStr"/>
+      <c r="AA5" t="inlineStr"/>
+      <c r="AB5" t="inlineStr"/>
+      <c r="AC5" t="inlineStr"/>
+      <c r="AD5" t="inlineStr"/>
+      <c r="AE5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -870,6 +942,14 @@
       <c r="U6" t="inlineStr"/>
       <c r="V6" t="inlineStr"/>
       <c r="W6" t="inlineStr"/>
+      <c r="X6" t="inlineStr"/>
+      <c r="Y6" t="inlineStr"/>
+      <c r="Z6" t="inlineStr"/>
+      <c r="AA6" t="inlineStr"/>
+      <c r="AB6" t="inlineStr"/>
+      <c r="AC6" t="inlineStr"/>
+      <c r="AD6" t="inlineStr"/>
+      <c r="AE6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -937,6 +1017,14 @@
       <c r="U7" t="inlineStr"/>
       <c r="V7" t="inlineStr"/>
       <c r="W7" t="inlineStr"/>
+      <c r="X7" t="inlineStr"/>
+      <c r="Y7" t="inlineStr"/>
+      <c r="Z7" t="inlineStr"/>
+      <c r="AA7" t="inlineStr"/>
+      <c r="AB7" t="inlineStr"/>
+      <c r="AC7" t="inlineStr"/>
+      <c r="AD7" t="inlineStr"/>
+      <c r="AE7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -1004,6 +1092,14 @@
       <c r="U8" t="inlineStr"/>
       <c r="V8" t="inlineStr"/>
       <c r="W8" t="inlineStr"/>
+      <c r="X8" t="inlineStr"/>
+      <c r="Y8" t="inlineStr"/>
+      <c r="Z8" t="inlineStr"/>
+      <c r="AA8" t="inlineStr"/>
+      <c r="AB8" t="inlineStr"/>
+      <c r="AC8" t="inlineStr"/>
+      <c r="AD8" t="inlineStr"/>
+      <c r="AE8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -1071,6 +1167,14 @@
       <c r="U9" t="inlineStr"/>
       <c r="V9" t="inlineStr"/>
       <c r="W9" t="inlineStr"/>
+      <c r="X9" t="inlineStr"/>
+      <c r="Y9" t="inlineStr"/>
+      <c r="Z9" t="inlineStr"/>
+      <c r="AA9" t="inlineStr"/>
+      <c r="AB9" t="inlineStr"/>
+      <c r="AC9" t="inlineStr"/>
+      <c r="AD9" t="inlineStr"/>
+      <c r="AE9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -1138,6 +1242,14 @@
       <c r="U10" t="inlineStr"/>
       <c r="V10" t="inlineStr"/>
       <c r="W10" t="inlineStr"/>
+      <c r="X10" t="inlineStr"/>
+      <c r="Y10" t="inlineStr"/>
+      <c r="Z10" t="inlineStr"/>
+      <c r="AA10" t="inlineStr"/>
+      <c r="AB10" t="inlineStr"/>
+      <c r="AC10" t="inlineStr"/>
+      <c r="AD10" t="inlineStr"/>
+      <c r="AE10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -1205,6 +1317,14 @@
       <c r="U11" t="inlineStr"/>
       <c r="V11" t="inlineStr"/>
       <c r="W11" t="inlineStr"/>
+      <c r="X11" t="inlineStr"/>
+      <c r="Y11" t="inlineStr"/>
+      <c r="Z11" t="inlineStr"/>
+      <c r="AA11" t="inlineStr"/>
+      <c r="AB11" t="inlineStr"/>
+      <c r="AC11" t="inlineStr"/>
+      <c r="AD11" t="inlineStr"/>
+      <c r="AE11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -1272,6 +1392,14 @@
       <c r="U12" t="inlineStr"/>
       <c r="V12" t="inlineStr"/>
       <c r="W12" t="inlineStr"/>
+      <c r="X12" t="inlineStr"/>
+      <c r="Y12" t="inlineStr"/>
+      <c r="Z12" t="inlineStr"/>
+      <c r="AA12" t="inlineStr"/>
+      <c r="AB12" t="inlineStr"/>
+      <c r="AC12" t="inlineStr"/>
+      <c r="AD12" t="inlineStr"/>
+      <c r="AE12" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -1339,6 +1467,14 @@
       <c r="U13" t="inlineStr"/>
       <c r="V13" t="inlineStr"/>
       <c r="W13" t="inlineStr"/>
+      <c r="X13" t="inlineStr"/>
+      <c r="Y13" t="inlineStr"/>
+      <c r="Z13" t="inlineStr"/>
+      <c r="AA13" t="inlineStr"/>
+      <c r="AB13" t="inlineStr"/>
+      <c r="AC13" t="inlineStr"/>
+      <c r="AD13" t="inlineStr"/>
+      <c r="AE13" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -1416,6 +1552,14 @@
       <c r="U14" t="inlineStr"/>
       <c r="V14" t="inlineStr"/>
       <c r="W14" t="inlineStr"/>
+      <c r="X14" t="inlineStr"/>
+      <c r="Y14" t="inlineStr"/>
+      <c r="Z14" t="inlineStr"/>
+      <c r="AA14" t="inlineStr"/>
+      <c r="AB14" t="inlineStr"/>
+      <c r="AC14" t="inlineStr"/>
+      <c r="AD14" t="inlineStr"/>
+      <c r="AE14" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -1493,6 +1637,14 @@
       <c r="U15" t="inlineStr"/>
       <c r="V15" t="inlineStr"/>
       <c r="W15" t="inlineStr"/>
+      <c r="X15" t="inlineStr"/>
+      <c r="Y15" t="inlineStr"/>
+      <c r="Z15" t="inlineStr"/>
+      <c r="AA15" t="inlineStr"/>
+      <c r="AB15" t="inlineStr"/>
+      <c r="AC15" t="inlineStr"/>
+      <c r="AD15" t="inlineStr"/>
+      <c r="AE15" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -1570,6 +1722,119 @@
       <c r="U16" t="inlineStr"/>
       <c r="V16" t="inlineStr"/>
       <c r="W16" t="inlineStr"/>
+      <c r="X16" t="inlineStr"/>
+      <c r="Y16" t="inlineStr"/>
+      <c r="Z16" t="inlineStr"/>
+      <c r="AA16" t="inlineStr"/>
+      <c r="AB16" t="inlineStr"/>
+      <c r="AC16" t="inlineStr"/>
+      <c r="AD16" t="inlineStr"/>
+      <c r="AE16" t="inlineStr"/>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>2026-09-14T15:10:22.390414+00:00</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>Bull</t>
+        </is>
+      </c>
+      <c r="E17" t="n">
+        <v>0.7366413617397212</v>
+      </c>
+      <c r="F17" t="n">
+        <v>0.1002546386571224</v>
+      </c>
+      <c r="G17" t="n">
+        <v>-0.836896000396844</v>
+      </c>
+      <c r="H17" t="n">
+        <v>0</v>
+      </c>
+      <c r="I17" t="b">
+        <v>0</v>
+      </c>
+      <c r="J17" t="n">
+        <v>1</v>
+      </c>
+      <c r="K17" t="n">
+        <v>0</v>
+      </c>
+      <c r="L17" t="n">
+        <v>0.8742411434848937</v>
+      </c>
+      <c r="M17" t="n">
+        <v>0.0615768919647658</v>
+      </c>
+      <c r="N17" t="n">
+        <v>0.06418196455034041</v>
+      </c>
+      <c r="O17" t="n">
+        <v>0.8742411434827887</v>
+      </c>
+      <c r="P17" t="n">
+        <v>0.0615768919658533</v>
+      </c>
+      <c r="Q17" t="n">
+        <v>0.064181964551358</v>
+      </c>
+      <c r="R17" t="inlineStr">
+        <is>
+          <t>FIN_PRE_EXDIV_KD</t>
+        </is>
+      </c>
+      <c r="S17" t="inlineStr">
+        <is>
+          <t>KD_APR15_MAY15_Klt30_T15</t>
+        </is>
+      </c>
+      <c r="T17" t="b">
+        <v>0</v>
+      </c>
+      <c r="U17" t="inlineStr"/>
+      <c r="V17" t="inlineStr"/>
+      <c r="W17" t="inlineStr"/>
+      <c r="X17" t="b">
+        <v>1</v>
+      </c>
+      <c r="Y17" t="b">
+        <v>1</v>
+      </c>
+      <c r="Z17" t="inlineStr">
+        <is>
+          <t>DH_dd06_vz1p0</t>
+        </is>
+      </c>
+      <c r="AA17" t="n">
+        <v>1</v>
+      </c>
+      <c r="AB17" t="n">
+        <v>0.8742411434848937</v>
+      </c>
+      <c r="AC17" t="n">
+        <v>0.0615768919647658</v>
+      </c>
+      <c r="AD17" t="n">
+        <v>0.06418196455034041</v>
+      </c>
+      <c r="AE17" t="inlineStr">
+        <is>
+          <t>ACCEPT Live cutover: DH_dd06 + FUSE_ADDITIVE</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -1582,7 +1847,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N16"/>
+  <dimension ref="A1:N17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2374,6 +2639,54 @@
         <v>0</v>
       </c>
       <c r="N16" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="B17" t="n">
+        <v>557445522.172183</v>
+      </c>
+      <c r="C17" t="n">
+        <v>1022.172182978364</v>
+      </c>
+      <c r="D17" t="n">
+        <v>0.8716272365175095</v>
+      </c>
+      <c r="E17" t="n">
+        <v>0.0589510520632536</v>
+      </c>
+      <c r="F17" t="n">
+        <v>0.0694198777473488</v>
+      </c>
+      <c r="G17" t="n">
+        <v>0.0104776600659046</v>
+      </c>
+      <c r="H17" t="n">
+        <v>0</v>
+      </c>
+      <c r="I17" t="n">
+        <v>0</v>
+      </c>
+      <c r="J17" t="b">
+        <v>1</v>
+      </c>
+      <c r="K17" t="n">
+        <v>0</v>
+      </c>
+      <c r="L17" t="inlineStr">
+        <is>
+          <t>E22_v2s_tw</t>
+        </is>
+      </c>
+      <c r="M17" t="n">
+        <v>0</v>
+      </c>
+      <c r="N17" t="n">
         <v>0</v>
       </c>
     </row>

</xml_diff>

<commit_message>
forward: update frozen E16 E18 E21 real-open ledgers (+ post-forward verify)
</commit_message>
<xml_diff>
--- a/forward/e21/E21_forward_dashboard.xlsx
+++ b/forward/e21/E21_forward_dashboard.xlsx
@@ -416,7 +416,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AE19"/>
+  <dimension ref="A1:AF20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -573,6 +573,11 @@
       <c r="AE1" t="inlineStr">
         <is>
           <t>live_cutover_ballot</t>
+        </is>
+      </c>
+      <c r="AF1" t="inlineStr">
+        <is>
+          <t>e45_stitch_rollback</t>
         </is>
       </c>
     </row>
@@ -650,6 +655,7 @@
       <c r="AC2" t="inlineStr"/>
       <c r="AD2" t="inlineStr"/>
       <c r="AE2" t="inlineStr"/>
+      <c r="AF2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -725,6 +731,7 @@
       <c r="AC3" t="inlineStr"/>
       <c r="AD3" t="inlineStr"/>
       <c r="AE3" t="inlineStr"/>
+      <c r="AF3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -800,6 +807,7 @@
       <c r="AC4" t="inlineStr"/>
       <c r="AD4" t="inlineStr"/>
       <c r="AE4" t="inlineStr"/>
+      <c r="AF4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -875,6 +883,7 @@
       <c r="AC5" t="inlineStr"/>
       <c r="AD5" t="inlineStr"/>
       <c r="AE5" t="inlineStr"/>
+      <c r="AF5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -950,6 +959,7 @@
       <c r="AC6" t="inlineStr"/>
       <c r="AD6" t="inlineStr"/>
       <c r="AE6" t="inlineStr"/>
+      <c r="AF6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -1025,6 +1035,7 @@
       <c r="AC7" t="inlineStr"/>
       <c r="AD7" t="inlineStr"/>
       <c r="AE7" t="inlineStr"/>
+      <c r="AF7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -1100,6 +1111,7 @@
       <c r="AC8" t="inlineStr"/>
       <c r="AD8" t="inlineStr"/>
       <c r="AE8" t="inlineStr"/>
+      <c r="AF8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -1175,6 +1187,7 @@
       <c r="AC9" t="inlineStr"/>
       <c r="AD9" t="inlineStr"/>
       <c r="AE9" t="inlineStr"/>
+      <c r="AF9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -1250,6 +1263,7 @@
       <c r="AC10" t="inlineStr"/>
       <c r="AD10" t="inlineStr"/>
       <c r="AE10" t="inlineStr"/>
+      <c r="AF10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -1325,6 +1339,7 @@
       <c r="AC11" t="inlineStr"/>
       <c r="AD11" t="inlineStr"/>
       <c r="AE11" t="inlineStr"/>
+      <c r="AF11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -1400,6 +1415,7 @@
       <c r="AC12" t="inlineStr"/>
       <c r="AD12" t="inlineStr"/>
       <c r="AE12" t="inlineStr"/>
+      <c r="AF12" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -1475,6 +1491,7 @@
       <c r="AC13" t="inlineStr"/>
       <c r="AD13" t="inlineStr"/>
       <c r="AE13" t="inlineStr"/>
+      <c r="AF13" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -1560,6 +1577,7 @@
       <c r="AC14" t="inlineStr"/>
       <c r="AD14" t="inlineStr"/>
       <c r="AE14" t="inlineStr"/>
+      <c r="AF14" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -1645,6 +1663,7 @@
       <c r="AC15" t="inlineStr"/>
       <c r="AD15" t="inlineStr"/>
       <c r="AE15" t="inlineStr"/>
+      <c r="AF15" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -1730,6 +1749,7 @@
       <c r="AC16" t="inlineStr"/>
       <c r="AD16" t="inlineStr"/>
       <c r="AE16" t="inlineStr"/>
+      <c r="AF16" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -1835,6 +1855,7 @@
           <t>ACCEPT Live cutover: DH_dd06 + FUSE_ADDITIVE</t>
         </is>
       </c>
+      <c r="AF17" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -1940,6 +1961,7 @@
           <t>ACCEPT Live cutover: DH_dd06 + FUSE_ADDITIVE</t>
         </is>
       </c>
+      <c r="AF18" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -2043,6 +2065,117 @@
       <c r="AE19" t="inlineStr">
         <is>
           <t>ACCEPT Live cutover: DH_dd06 + FUSE_ADDITIVE</t>
+        </is>
+      </c>
+      <c r="AF19" t="inlineStr"/>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>2026-09-21</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>2026-09-21T14:20:59.820566+00:00</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>2026-09-21</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>Bull</t>
+        </is>
+      </c>
+      <c r="E20" t="n">
+        <v>0.5555474267120171</v>
+      </c>
+      <c r="F20" t="n">
+        <v>-0.2321322128005977</v>
+      </c>
+      <c r="G20" t="n">
+        <v>-0.3234152139114191</v>
+      </c>
+      <c r="H20" t="n">
+        <v>1</v>
+      </c>
+      <c r="I20" t="b">
+        <v>0</v>
+      </c>
+      <c r="J20" t="n">
+        <v>2</v>
+      </c>
+      <c r="K20" t="n">
+        <v>0</v>
+      </c>
+      <c r="L20" t="n">
+        <v>0.8806808576136702</v>
+      </c>
+      <c r="M20" t="n">
+        <v>0.0661794982823404</v>
+      </c>
+      <c r="N20" t="n">
+        <v>0.0531396441039893</v>
+      </c>
+      <c r="O20" t="n">
+        <v>0.8806808576120915</v>
+      </c>
+      <c r="P20" t="n">
+        <v>0.066179498283156</v>
+      </c>
+      <c r="Q20" t="n">
+        <v>0.0531396441047524</v>
+      </c>
+      <c r="R20" t="inlineStr">
+        <is>
+          <t>FIN_PRE_EXDIV_KD</t>
+        </is>
+      </c>
+      <c r="S20" t="inlineStr">
+        <is>
+          <t>KD_APR15_MAY15_Klt30_T15</t>
+        </is>
+      </c>
+      <c r="T20" t="b">
+        <v>0</v>
+      </c>
+      <c r="U20" t="inlineStr"/>
+      <c r="V20" t="inlineStr"/>
+      <c r="W20" t="inlineStr"/>
+      <c r="X20" t="b">
+        <v>1</v>
+      </c>
+      <c r="Y20" t="b">
+        <v>1</v>
+      </c>
+      <c r="Z20" t="inlineStr">
+        <is>
+          <t>DH_dd06_vz1p0</t>
+        </is>
+      </c>
+      <c r="AA20" t="n">
+        <v>1</v>
+      </c>
+      <c r="AB20" t="n">
+        <v>0.8806808576136702</v>
+      </c>
+      <c r="AC20" t="n">
+        <v>0.0661794982823404</v>
+      </c>
+      <c r="AD20" t="n">
+        <v>0.0531396441039893</v>
+      </c>
+      <c r="AE20" t="inlineStr">
+        <is>
+          <t>ACCEPT Live cutover: DH_dd06 + FUSE_ADDITIVE</t>
+        </is>
+      </c>
+      <c r="AF20" t="inlineStr">
+        <is>
+          <t>ACCEPT_2026-09-09_DROP_E45_A05</t>
         </is>
       </c>
     </row>
@@ -2057,7 +2190,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N19"/>
+  <dimension ref="A1:Q20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2131,6 +2264,21 @@
           <t>e22_stock_shares_added</t>
         </is>
       </c>
+      <c r="O1" t="inlineStr">
+        <is>
+          <t>e22_receivable_credit</t>
+        </is>
+      </c>
+      <c r="P1" t="inlineStr">
+        <is>
+          <t>e22_receivable_settled</t>
+        </is>
+      </c>
+      <c r="Q1" t="inlineStr">
+        <is>
+          <t>e22_receivable_balance</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -2179,6 +2327,9 @@
       <c r="N2" t="n">
         <v>0</v>
       </c>
+      <c r="O2" t="inlineStr"/>
+      <c r="P2" t="inlineStr"/>
+      <c r="Q2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -2227,6 +2378,9 @@
       <c r="N3" t="n">
         <v>0</v>
       </c>
+      <c r="O3" t="inlineStr"/>
+      <c r="P3" t="inlineStr"/>
+      <c r="Q3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -2275,6 +2429,9 @@
       <c r="N4" t="n">
         <v>0</v>
       </c>
+      <c r="O4" t="inlineStr"/>
+      <c r="P4" t="inlineStr"/>
+      <c r="Q4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -2323,6 +2480,9 @@
       <c r="N5" t="n">
         <v>0</v>
       </c>
+      <c r="O5" t="inlineStr"/>
+      <c r="P5" t="inlineStr"/>
+      <c r="Q5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -2371,6 +2531,9 @@
       <c r="N6" t="n">
         <v>0</v>
       </c>
+      <c r="O6" t="inlineStr"/>
+      <c r="P6" t="inlineStr"/>
+      <c r="Q6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -2419,6 +2582,9 @@
       <c r="N7" t="n">
         <v>0</v>
       </c>
+      <c r="O7" t="inlineStr"/>
+      <c r="P7" t="inlineStr"/>
+      <c r="Q7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -2467,6 +2633,9 @@
       <c r="N8" t="n">
         <v>0</v>
       </c>
+      <c r="O8" t="inlineStr"/>
+      <c r="P8" t="inlineStr"/>
+      <c r="Q8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -2515,6 +2684,9 @@
       <c r="N9" t="n">
         <v>0</v>
       </c>
+      <c r="O9" t="inlineStr"/>
+      <c r="P9" t="inlineStr"/>
+      <c r="Q9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -2563,6 +2735,9 @@
       <c r="N10" t="n">
         <v>0</v>
       </c>
+      <c r="O10" t="inlineStr"/>
+      <c r="P10" t="inlineStr"/>
+      <c r="Q10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -2611,6 +2786,9 @@
       <c r="N11" t="n">
         <v>0</v>
       </c>
+      <c r="O11" t="inlineStr"/>
+      <c r="P11" t="inlineStr"/>
+      <c r="Q11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -2659,6 +2837,9 @@
       <c r="N12" t="n">
         <v>0</v>
       </c>
+      <c r="O12" t="inlineStr"/>
+      <c r="P12" t="inlineStr"/>
+      <c r="Q12" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -2707,6 +2888,9 @@
       <c r="N13" t="n">
         <v>0</v>
       </c>
+      <c r="O13" t="inlineStr"/>
+      <c r="P13" t="inlineStr"/>
+      <c r="Q13" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -2755,6 +2939,9 @@
       <c r="N14" t="n">
         <v>0</v>
       </c>
+      <c r="O14" t="inlineStr"/>
+      <c r="P14" t="inlineStr"/>
+      <c r="Q14" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -2803,6 +2990,9 @@
       <c r="N15" t="n">
         <v>0</v>
       </c>
+      <c r="O15" t="inlineStr"/>
+      <c r="P15" t="inlineStr"/>
+      <c r="Q15" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -2851,6 +3041,9 @@
       <c r="N16" t="n">
         <v>0</v>
       </c>
+      <c r="O16" t="inlineStr"/>
+      <c r="P16" t="inlineStr"/>
+      <c r="Q16" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -2899,6 +3092,9 @@
       <c r="N17" t="n">
         <v>0</v>
       </c>
+      <c r="O17" t="inlineStr"/>
+      <c r="P17" t="inlineStr"/>
+      <c r="Q17" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -2947,6 +3143,9 @@
       <c r="N18" t="n">
         <v>0</v>
       </c>
+      <c r="O18" t="inlineStr"/>
+      <c r="P18" t="inlineStr"/>
+      <c r="Q18" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -2993,6 +3192,66 @@
         <v>0</v>
       </c>
       <c r="N19" t="n">
+        <v>0</v>
+      </c>
+      <c r="O19" t="inlineStr"/>
+      <c r="P19" t="inlineStr"/>
+      <c r="Q19" t="inlineStr"/>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>2026-09-21</t>
+        </is>
+      </c>
+      <c r="B20" t="n">
+        <v>555499915.5135857</v>
+      </c>
+      <c r="C20" t="n">
+        <v>50415.51358572836</v>
+      </c>
+      <c r="D20" t="n">
+        <v>0.8753941025362896</v>
+      </c>
+      <c r="E20" t="n">
+        <v>0.0645805678779129</v>
+      </c>
+      <c r="F20" t="n">
+        <v>0.05993457257184</v>
+      </c>
+      <c r="G20" t="n">
+        <v>0.0136806139496588</v>
+      </c>
+      <c r="H20" t="n">
+        <v>0</v>
+      </c>
+      <c r="I20" t="n">
+        <v>0</v>
+      </c>
+      <c r="J20" t="b">
+        <v>1</v>
+      </c>
+      <c r="K20" t="n">
+        <v>0</v>
+      </c>
+      <c r="L20" t="inlineStr">
+        <is>
+          <t>E22_v3_recv_pay_effdelay</t>
+        </is>
+      </c>
+      <c r="M20" t="n">
+        <v>0</v>
+      </c>
+      <c r="N20" t="n">
+        <v>0</v>
+      </c>
+      <c r="O20" t="n">
+        <v>0</v>
+      </c>
+      <c r="P20" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q20" t="n">
         <v>0</v>
       </c>
     </row>

</xml_diff>